<commit_message>
Fix PSRAM footprint (RP2350)
</commit_message>
<xml_diff>
--- a/pcb/esp32p4/mainboard/pcb assembly JLC/p2_pcb_esp32p4_v1_4_bom_JLC.xlsx
+++ b/pcb/esp32p4/mainboard/pcb assembly JLC/p2_pcb_esp32p4_v1_4_bom_JLC.xlsx
@@ -5,7 +5,7 @@
   <workbookPr defaultThemeVersion="153222"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Daniel\Desktop\Proj_i\picoheld2_hardware\picoheld2_public\picoheld2\pcb\esp32p4\mainboard\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Daniel\Desktop\Proj_i\picoheld2_hardware\picoheld2_public\picoheld2\pcb\esp32p4\mainboard\pcb assembly JLC\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -54,45 +54,30 @@
     <t>C17767</t>
   </si>
   <si>
-    <t>33R</t>
-  </si>
-  <si>
     <t>R7,R8</t>
   </si>
   <si>
     <t>C17634</t>
   </si>
   <si>
-    <t>10k</t>
-  </si>
-  <si>
     <t>R9,R3,R19,R13,R23,R14,R16,R33,R15,R17,R20,R4,R22,R31</t>
   </si>
   <si>
     <t>C17414</t>
   </si>
   <si>
-    <t>100k</t>
-  </si>
-  <si>
     <t>R12,R32,R10,R26,R11,R5,R6</t>
   </si>
   <si>
     <t>C25611</t>
   </si>
   <si>
-    <t>1.65k</t>
-  </si>
-  <si>
     <t>R18</t>
   </si>
   <si>
     <t>C17393</t>
   </si>
   <si>
-    <t>30k</t>
-  </si>
-  <si>
     <t>R21,R24</t>
   </si>
   <si>
@@ -108,18 +93,12 @@
     <t>C53884</t>
   </si>
   <si>
-    <t>5.1k</t>
-  </si>
-  <si>
     <t>R25,R28</t>
   </si>
   <si>
     <t>C26023</t>
   </si>
   <si>
-    <t>20k</t>
-  </si>
-  <si>
     <t>R30</t>
   </si>
   <si>
@@ -132,30 +111,18 @@
     <t>C13585</t>
   </si>
   <si>
-    <t>C11,C2,C5,C4</t>
-  </si>
-  <si>
     <t>C_0805_2012Metric</t>
   </si>
   <si>
     <t>C1713</t>
   </si>
   <si>
-    <t>22uF</t>
-  </si>
-  <si>
     <t>C7</t>
   </si>
   <si>
     <t>C1859</t>
   </si>
   <si>
-    <t>10uF</t>
-  </si>
-  <si>
-    <t>1uF</t>
-  </si>
-  <si>
     <t>C8,C1,C10,C24,C25</t>
   </si>
   <si>
@@ -168,18 +135,12 @@
     <t>C26</t>
   </si>
   <si>
-    <t>100nF</t>
-  </si>
-  <si>
     <t>C13,C12</t>
   </si>
   <si>
     <t>C28233</t>
   </si>
   <si>
-    <t>MBR120VLSFT1G</t>
-  </si>
-  <si>
     <t>D3,D1</t>
   </si>
   <si>
@@ -189,9 +150,6 @@
     <t>C223608</t>
   </si>
   <si>
-    <t>SCHOTTKY DIODE SS24 2A 40V SMA SR240 DO-214AC</t>
-  </si>
-  <si>
     <t>D2</t>
   </si>
   <si>
@@ -201,9 +159,6 @@
     <t>C50645</t>
   </si>
   <si>
-    <t>3.3uH (NRS5030T3R3MMGJ)</t>
-  </si>
-  <si>
     <t>L1</t>
   </si>
   <si>
@@ -213,9 +168,6 @@
     <t>C222937</t>
   </si>
   <si>
-    <t>DMG2305UX</t>
-  </si>
-  <si>
     <t>T1</t>
   </si>
   <si>
@@ -225,18 +177,12 @@
     <t>C150470</t>
   </si>
   <si>
-    <t>FDN340P</t>
-  </si>
-  <si>
     <t>Q1</t>
   </si>
   <si>
     <t>C75469</t>
   </si>
   <si>
-    <t>sdb628</t>
-  </si>
-  <si>
     <t>U1</t>
   </si>
   <si>
@@ -246,9 +192,6 @@
     <t>C30197563</t>
   </si>
   <si>
-    <t>AO3401</t>
-  </si>
-  <si>
     <t>U2</t>
   </si>
   <si>
@@ -258,9 +201,6 @@
     <t>C15127</t>
   </si>
   <si>
-    <t>NS4168</t>
-  </si>
-  <si>
     <t>U3</t>
   </si>
   <si>
@@ -270,9 +210,6 @@
     <t>C910588</t>
   </si>
   <si>
-    <t>TPS22810TDBVRQ1</t>
-  </si>
-  <si>
     <t>U4</t>
   </si>
   <si>
@@ -282,36 +219,21 @@
     <t>C2877634</t>
   </si>
   <si>
-    <t>XC6222B331MR-G</t>
-  </si>
-  <si>
     <t>U5</t>
   </si>
   <si>
     <t>SOT-25_TOR</t>
   </si>
   <si>
-    <t>C9900057694</t>
-  </si>
-  <si>
-    <t>AO3402</t>
-  </si>
-  <si>
     <t>U7,U6</t>
   </si>
   <si>
     <t>C14385</t>
   </si>
   <si>
-    <t>TP4054</t>
-  </si>
-  <si>
     <t>U8</t>
   </si>
   <si>
-    <t>C32574</t>
-  </si>
-  <si>
     <t>WT0132P4_SOM</t>
   </si>
   <si>
@@ -321,9 +243,6 @@
     <t>C9900155824</t>
   </si>
   <si>
-    <t>XC6206P182MR</t>
-  </si>
-  <si>
     <t>U10</t>
   </si>
   <si>
@@ -333,27 +252,18 @@
     <t>C21659</t>
   </si>
   <si>
-    <t>pj242</t>
-  </si>
-  <si>
     <t>J1</t>
   </si>
   <si>
     <t>C431536</t>
   </si>
   <si>
-    <t>0.5K-DX-40PWBG</t>
-  </si>
-  <si>
     <t>J2</t>
   </si>
   <si>
     <t>FH12-30S-0.5SH</t>
   </si>
   <si>
-    <t>USB_B_Micro</t>
-  </si>
-  <si>
     <t>J4</t>
   </si>
   <si>
@@ -363,9 +273,6 @@
     <t>C2988369</t>
   </si>
   <si>
-    <t>Micro_SD_Card_Det1</t>
-  </si>
-  <si>
     <t>J5</t>
   </si>
   <si>
@@ -375,9 +282,6 @@
     <t>C2889258</t>
   </si>
   <si>
-    <t>Conn_01x05_Socket</t>
-  </si>
-  <si>
     <t>J7</t>
   </si>
   <si>
@@ -387,9 +291,6 @@
     <t>C262230</t>
   </si>
   <si>
-    <t>SW_Push</t>
-  </si>
-  <si>
     <t>SW9</t>
   </si>
   <si>
@@ -399,22 +300,121 @@
     <t>C2886886</t>
   </si>
   <si>
-    <t>BTN_ST, SEL</t>
-  </si>
-  <si>
     <t>SW10, SW11</t>
   </si>
   <si>
     <t>SW_SPST_TL3342</t>
   </si>
   <si>
-    <t>C6,C3,C9</t>
-  </si>
-  <si>
     <t>C506793</t>
   </si>
   <si>
     <t>C2886894</t>
+  </si>
+  <si>
+    <t>SHOU HAN PJ-242</t>
+  </si>
+  <si>
+    <t>Hirose FH12-30S-0.5SH(55)</t>
+  </si>
+  <si>
+    <t>G-Switch GT-USB-7010ASV</t>
+  </si>
+  <si>
+    <t>Yuandi  TF-01A</t>
+  </si>
+  <si>
+    <t>Jushuo AFC07-S05ECC-00</t>
+  </si>
+  <si>
+    <t>E-Switch TL3330AF260QG</t>
+  </si>
+  <si>
+    <t>E-Switch TL3342F260QG</t>
+  </si>
+  <si>
+    <t>Torex Semicon XC6206P182MR</t>
+  </si>
+  <si>
+    <t>AO Semi AO3402</t>
+  </si>
+  <si>
+    <t>TI TPS22810TDBVRQ1</t>
+  </si>
+  <si>
+    <t>Shenzhen Nsiway Tech NS4168</t>
+  </si>
+  <si>
+    <t>AO Semi AO3401</t>
+  </si>
+  <si>
+    <t>MSKSEMI SDB628</t>
+  </si>
+  <si>
+    <t>onsemi FDN340P</t>
+  </si>
+  <si>
+    <t>Diodes Inc. DMG2305UX-7</t>
+  </si>
+  <si>
+    <t>Taiyo Yuden NRS5030T3R3MMGJ (3.3 uH)</t>
+  </si>
+  <si>
+    <t>MDD SS24 (SCHOTTKY DIODE SS24 2A 40V SMA SR240 DO-214AC)</t>
+  </si>
+  <si>
+    <t>onsemi MBR120VLSFT1G</t>
+  </si>
+  <si>
+    <t>33R 1%</t>
+  </si>
+  <si>
+    <t>10k 1%</t>
+  </si>
+  <si>
+    <t>100k 1%</t>
+  </si>
+  <si>
+    <t>1.65k 1%</t>
+  </si>
+  <si>
+    <t>30k 1%</t>
+  </si>
+  <si>
+    <t>5.1k 1%</t>
+  </si>
+  <si>
+    <t>20k 1%</t>
+  </si>
+  <si>
+    <t>10uF 10%</t>
+  </si>
+  <si>
+    <t>22uF 10%</t>
+  </si>
+  <si>
+    <t>1uF 10%</t>
+  </si>
+  <si>
+    <t>100nF 10%</t>
+  </si>
+  <si>
+    <t>C12044</t>
+  </si>
+  <si>
+    <t>TOPPOWER TP4057-42-SOT26-R</t>
+  </si>
+  <si>
+    <t>Torex Semicon XC6220B331MR-G</t>
+  </si>
+  <si>
+    <t>C86534</t>
+  </si>
+  <si>
+    <t>C11,C9,C2,C5,C4</t>
+  </si>
+  <si>
+    <t>C6,C3</t>
   </si>
 </sst>
 </file>
@@ -898,8 +898,11 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="17" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20 % - Akzent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1224,6 +1227,7 @@
   <dimension ref="A1:D38"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
+    <col min="1" max="1" width="32.62890625" customWidth="1"/>
     <col min="3" max="3" width="34.7890625" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1271,483 +1275,483 @@
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A4" t="s">
+        <v>115</v>
+      </c>
+      <c r="B4" t="s">
         <v>11</v>
-      </c>
-      <c r="B4" t="s">
-        <v>12</v>
       </c>
       <c r="C4" t="s">
         <v>6</v>
       </c>
       <c r="D4" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A5" t="s">
-        <v>14</v>
+        <v>116</v>
       </c>
       <c r="B5" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="C5" t="s">
         <v>6</v>
       </c>
       <c r="D5" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A6" t="s">
-        <v>17</v>
+        <v>117</v>
       </c>
       <c r="B6" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="C6" t="s">
         <v>6</v>
       </c>
       <c r="D6" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A7" t="s">
-        <v>20</v>
+        <v>118</v>
       </c>
       <c r="B7" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="C7" t="s">
         <v>6</v>
       </c>
       <c r="D7" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A8" t="s">
-        <v>23</v>
+        <v>119</v>
       </c>
       <c r="B8" t="s">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="C8" t="s">
         <v>6</v>
       </c>
       <c r="D8" t="s">
-        <v>25</v>
+        <v>20</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A9" t="s">
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="B9" t="s">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="C9" t="s">
         <v>6</v>
       </c>
       <c r="D9" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A10" t="s">
-        <v>29</v>
+        <v>120</v>
       </c>
       <c r="B10" t="s">
-        <v>30</v>
+        <v>24</v>
       </c>
       <c r="C10" t="s">
         <v>6</v>
       </c>
       <c r="D10" t="s">
-        <v>31</v>
+        <v>25</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A11" t="s">
-        <v>32</v>
+        <v>121</v>
       </c>
       <c r="B11" t="s">
-        <v>33</v>
+        <v>26</v>
       </c>
       <c r="C11" t="s">
         <v>6</v>
       </c>
       <c r="D11" t="s">
-        <v>34</v>
+        <v>27</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A12" t="s">
-        <v>43</v>
+        <v>122</v>
       </c>
       <c r="B12" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="C12" t="s">
-        <v>35</v>
+        <v>28</v>
       </c>
       <c r="D12" t="s">
-        <v>36</v>
+        <v>29</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A13" t="s">
-        <v>43</v>
+        <v>122</v>
       </c>
       <c r="B13" t="s">
-        <v>37</v>
+        <v>130</v>
       </c>
       <c r="C13" t="s">
-        <v>38</v>
+        <v>30</v>
       </c>
       <c r="D13" t="s">
-        <v>39</v>
+        <v>31</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A14" t="s">
-        <v>40</v>
+        <v>123</v>
       </c>
       <c r="B14" t="s">
-        <v>41</v>
+        <v>32</v>
       </c>
       <c r="C14" t="s">
-        <v>35</v>
+        <v>28</v>
       </c>
       <c r="D14" t="s">
-        <v>42</v>
+        <v>33</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A15" t="s">
-        <v>44</v>
+        <v>124</v>
       </c>
       <c r="B15" t="s">
-        <v>45</v>
+        <v>34</v>
       </c>
       <c r="C15" t="s">
-        <v>38</v>
+        <v>30</v>
       </c>
       <c r="D15" t="s">
-        <v>46</v>
+        <v>35</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A16" t="s">
-        <v>47</v>
+        <v>36</v>
       </c>
       <c r="B16" t="s">
-        <v>48</v>
+        <v>37</v>
       </c>
       <c r="C16" t="s">
-        <v>38</v>
+        <v>30</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A17" t="s">
-        <v>49</v>
+        <v>125</v>
       </c>
       <c r="B17" t="s">
-        <v>50</v>
+        <v>38</v>
       </c>
       <c r="C17" t="s">
-        <v>38</v>
+        <v>30</v>
       </c>
       <c r="D17" t="s">
-        <v>51</v>
+        <v>39</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A18" t="s">
-        <v>52</v>
+        <v>114</v>
       </c>
       <c r="B18" t="s">
-        <v>53</v>
+        <v>40</v>
       </c>
       <c r="C18" t="s">
-        <v>54</v>
+        <v>41</v>
       </c>
       <c r="D18" t="s">
-        <v>55</v>
+        <v>42</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A19" t="s">
-        <v>56</v>
+        <v>113</v>
       </c>
       <c r="B19" t="s">
-        <v>57</v>
+        <v>43</v>
       </c>
       <c r="C19" t="s">
-        <v>58</v>
+        <v>44</v>
       </c>
       <c r="D19" t="s">
-        <v>59</v>
+        <v>45</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A20" t="s">
-        <v>60</v>
+        <v>112</v>
       </c>
       <c r="B20" t="s">
-        <v>61</v>
+        <v>46</v>
       </c>
       <c r="C20" t="s">
-        <v>62</v>
+        <v>47</v>
       </c>
       <c r="D20" t="s">
-        <v>63</v>
+        <v>48</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.55000000000000004">
-      <c r="A21" t="s">
-        <v>64</v>
+      <c r="A21" s="1" t="s">
+        <v>111</v>
       </c>
       <c r="B21" t="s">
-        <v>65</v>
+        <v>49</v>
       </c>
       <c r="C21" t="s">
-        <v>66</v>
+        <v>50</v>
       </c>
       <c r="D21" t="s">
-        <v>67</v>
+        <v>51</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A22" t="s">
-        <v>68</v>
+        <v>110</v>
       </c>
       <c r="B22" t="s">
-        <v>69</v>
+        <v>52</v>
       </c>
       <c r="C22" t="s">
-        <v>66</v>
+        <v>50</v>
       </c>
       <c r="D22" t="s">
-        <v>70</v>
+        <v>53</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A23" t="s">
-        <v>71</v>
+        <v>109</v>
       </c>
       <c r="B23" t="s">
-        <v>72</v>
+        <v>54</v>
       </c>
       <c r="C23" t="s">
-        <v>73</v>
+        <v>55</v>
       </c>
       <c r="D23" t="s">
-        <v>74</v>
+        <v>56</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A24" t="s">
-        <v>75</v>
+        <v>108</v>
       </c>
       <c r="B24" t="s">
-        <v>76</v>
+        <v>57</v>
       </c>
       <c r="C24" t="s">
-        <v>77</v>
+        <v>58</v>
       </c>
       <c r="D24" t="s">
-        <v>78</v>
+        <v>59</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A25" t="s">
-        <v>79</v>
+        <v>107</v>
       </c>
       <c r="B25" t="s">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="C25" t="s">
-        <v>81</v>
+        <v>61</v>
       </c>
       <c r="D25" t="s">
-        <v>82</v>
+        <v>62</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A26" t="s">
-        <v>83</v>
+        <v>106</v>
       </c>
       <c r="B26" t="s">
-        <v>84</v>
+        <v>63</v>
       </c>
       <c r="C26" t="s">
-        <v>85</v>
+        <v>64</v>
       </c>
       <c r="D26" t="s">
-        <v>86</v>
+        <v>65</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.55000000000000004">
-      <c r="A27" t="s">
-        <v>87</v>
+      <c r="A27" s="1" t="s">
+        <v>128</v>
       </c>
       <c r="B27" t="s">
-        <v>88</v>
+        <v>66</v>
       </c>
       <c r="C27" t="s">
-        <v>89</v>
+        <v>67</v>
       </c>
       <c r="D27" t="s">
-        <v>90</v>
+        <v>129</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A28" t="s">
-        <v>91</v>
+        <v>105</v>
       </c>
       <c r="B28" t="s">
-        <v>92</v>
+        <v>68</v>
       </c>
       <c r="C28" t="s">
-        <v>77</v>
+        <v>58</v>
       </c>
       <c r="D28" t="s">
-        <v>93</v>
+        <v>69</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A29" t="s">
-        <v>94</v>
+        <v>127</v>
       </c>
       <c r="B29" t="s">
-        <v>95</v>
+        <v>70</v>
       </c>
       <c r="C29" t="s">
-        <v>73</v>
+        <v>55</v>
       </c>
       <c r="D29" t="s">
-        <v>96</v>
+        <v>126</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A30" t="s">
-        <v>97</v>
+        <v>71</v>
       </c>
       <c r="B30" t="s">
-        <v>98</v>
+        <v>72</v>
       </c>
       <c r="D30" t="s">
-        <v>99</v>
+        <v>73</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.55000000000000004">
-      <c r="A31" t="s">
-        <v>100</v>
+      <c r="A31" s="1" t="s">
+        <v>104</v>
       </c>
       <c r="B31" t="s">
-        <v>101</v>
+        <v>74</v>
       </c>
       <c r="C31" t="s">
-        <v>102</v>
+        <v>75</v>
       </c>
       <c r="D31" t="s">
-        <v>103</v>
+        <v>76</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A32" t="s">
-        <v>104</v>
+        <v>97</v>
       </c>
       <c r="B32" t="s">
-        <v>105</v>
+        <v>77</v>
       </c>
       <c r="D32" t="s">
-        <v>106</v>
+        <v>78</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A33" t="s">
-        <v>107</v>
+        <v>98</v>
       </c>
       <c r="B33" t="s">
-        <v>108</v>
+        <v>79</v>
       </c>
       <c r="C33" t="s">
-        <v>109</v>
+        <v>80</v>
       </c>
       <c r="D33" t="s">
-        <v>130</v>
+        <v>95</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.55000000000000004">
-      <c r="A34" t="s">
-        <v>110</v>
+      <c r="A34" s="1" t="s">
+        <v>99</v>
       </c>
       <c r="B34" t="s">
-        <v>111</v>
+        <v>81</v>
       </c>
       <c r="C34" t="s">
-        <v>112</v>
+        <v>82</v>
       </c>
       <c r="D34" t="s">
-        <v>113</v>
+        <v>83</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A35" t="s">
-        <v>114</v>
+        <v>100</v>
       </c>
       <c r="B35" t="s">
-        <v>115</v>
+        <v>84</v>
       </c>
       <c r="C35" t="s">
-        <v>116</v>
+        <v>85</v>
       </c>
       <c r="D35" t="s">
-        <v>117</v>
+        <v>86</v>
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A36" t="s">
-        <v>118</v>
+        <v>101</v>
       </c>
       <c r="B36" t="s">
-        <v>119</v>
+        <v>87</v>
       </c>
       <c r="C36" t="s">
-        <v>120</v>
+        <v>88</v>
       </c>
       <c r="D36" t="s">
-        <v>121</v>
+        <v>89</v>
       </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A37" t="s">
-        <v>122</v>
+        <v>102</v>
       </c>
       <c r="B37" t="s">
-        <v>123</v>
+        <v>90</v>
       </c>
       <c r="C37" t="s">
-        <v>124</v>
+        <v>91</v>
       </c>
       <c r="D37" t="s">
-        <v>125</v>
+        <v>92</v>
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A38" t="s">
-        <v>126</v>
+        <v>103</v>
       </c>
       <c r="B38" t="s">
-        <v>127</v>
+        <v>93</v>
       </c>
       <c r="C38" t="s">
-        <v>128</v>
+        <v>94</v>
       </c>
       <c r="D38" t="s">
-        <v>131</v>
+        <v>96</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fix board cannot start without battery
</commit_message>
<xml_diff>
--- a/pcb/esp32p4/mainboard/pcb assembly JLC/p2_pcb_esp32p4_v1_4_bom_JLC.xlsx
+++ b/pcb/esp32p4/mainboard/pcb assembly JLC/p2_pcb_esp32p4_v1_4_bom_JLC.xlsx
@@ -60,9 +60,6 @@
     <t>C17634</t>
   </si>
   <si>
-    <t>R9,R3,R19,R13,R23,R14,R16,R33,R15,R17,R20,R4,R22,R31</t>
-  </si>
-  <si>
     <t>C17414</t>
   </si>
   <si>
@@ -78,9 +75,6 @@
     <t>C17393</t>
   </si>
   <si>
-    <t>R21,R24</t>
-  </si>
-  <si>
     <t>C17621</t>
   </si>
   <si>
@@ -99,9 +93,6 @@
     <t>C26023</t>
   </si>
   <si>
-    <t>R30</t>
-  </si>
-  <si>
     <t>C4328</t>
   </si>
   <si>
@@ -415,6 +406,15 @@
   </si>
   <si>
     <t>C6,C3</t>
+  </si>
+  <si>
+    <t>R21</t>
+  </si>
+  <si>
+    <t>R9,R3,R19,R13,R14,R16,R33,R15,R17,R20,R4,R22,R31</t>
+  </si>
+  <si>
+    <t>R23,R24,R30</t>
   </si>
 </sst>
 </file>
@@ -1275,7 +1275,7 @@
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A4" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="B4" t="s">
         <v>11</v>
@@ -1289,469 +1289,469 @@
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A5" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="B5" t="s">
-        <v>13</v>
+        <v>130</v>
       </c>
       <c r="C5" t="s">
         <v>6</v>
       </c>
       <c r="D5" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A6" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="B6" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C6" t="s">
         <v>6</v>
       </c>
       <c r="D6" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A7" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="B7" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C7" t="s">
         <v>6</v>
       </c>
       <c r="D7" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A8" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="B8" t="s">
-        <v>19</v>
+        <v>129</v>
       </c>
       <c r="C8" t="s">
         <v>6</v>
       </c>
       <c r="D8" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A9" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B9" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="C9" t="s">
         <v>6</v>
       </c>
       <c r="D9" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A10" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="B10" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="C10" t="s">
         <v>6</v>
       </c>
       <c r="D10" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A11" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="B11" t="s">
-        <v>26</v>
+        <v>131</v>
       </c>
       <c r="C11" t="s">
         <v>6</v>
       </c>
       <c r="D11" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A12" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="B12" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="C12" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="D12" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A13" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="B13" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
       <c r="C13" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="D13" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A14" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="B14" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="C14" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="D14" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A15" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="B15" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="C15" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="D15" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A16" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="B16" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="C16" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A17" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="B17" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="C17" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="D17" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A18" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="B18" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="C18" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="D18" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A19" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="B19" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="C19" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="D19" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A20" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="B20" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="C20" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="D20" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A21" s="1" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="B21" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="C21" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="D21" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A22" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="B22" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="C22" t="s">
+        <v>47</v>
+      </c>
+      <c r="D22" t="s">
         <v>50</v>
-      </c>
-      <c r="D22" t="s">
-        <v>53</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A23" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="B23" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="C23" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="D23" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A24" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="B24" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="C24" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="D24" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A25" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="B25" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="C25" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="D25" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A26" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="B26" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="C26" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="D26" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A27" s="1" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="B27" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="C27" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="D27" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A28" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="B28" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="C28" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="D28" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A29" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="B29" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="C29" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="D29" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A30" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="B30" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="D30" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A31" s="1" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="B31" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="C31" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="D31" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A32" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="B32" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="D32" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A33" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="B33" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="C33" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="D33" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A34" s="1" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="B34" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="C34" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="D34" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A35" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="B35" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="C35" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="D35" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A36" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="B36" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="C36" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="D36" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A37" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="B37" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="C37" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="D37" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A38" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="B38" t="s">
+        <v>90</v>
+      </c>
+      <c r="C38" t="s">
+        <v>91</v>
+      </c>
+      <c r="D38" t="s">
         <v>93</v>
-      </c>
-      <c r="C38" t="s">
-        <v>94</v>
-      </c>
-      <c r="D38" t="s">
-        <v>96</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fix inductor part (was too tall)
</commit_message>
<xml_diff>
--- a/pcb/esp32p4/mainboard/pcb assembly JLC/p2_pcb_esp32p4_v1_4_bom_JLC.xlsx
+++ b/pcb/esp32p4/mainboard/pcb assembly JLC/p2_pcb_esp32p4_v1_4_bom_JLC.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="149" uniqueCount="132">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="151" uniqueCount="134">
   <si>
     <t>Comment</t>
   </si>
@@ -153,12 +153,6 @@
     <t>L1</t>
   </si>
   <si>
-    <t>L_APV_ANR5012</t>
-  </si>
-  <si>
-    <t>C222937</t>
-  </si>
-  <si>
     <t>T1</t>
   </si>
   <si>
@@ -348,9 +342,6 @@
     <t>Diodes Inc. DMG2305UX-7</t>
   </si>
   <si>
-    <t>Taiyo Yuden NRS5030T3R3MMGJ (3.3 uH)</t>
-  </si>
-  <si>
     <t>MDD SS24 (SCHOTTKY DIODE SS24 2A 40V SMA SR240 DO-214AC)</t>
   </si>
   <si>
@@ -415,6 +406,21 @@
   </si>
   <si>
     <t>R23,R24,R30</t>
+  </si>
+  <si>
+    <t>J6</t>
+  </si>
+  <si>
+    <t>GH 1.25 (LiPo connector)</t>
+  </si>
+  <si>
+    <t>C668614</t>
+  </si>
+  <si>
+    <t>SWPA5020S3R3MT (3.3 uH, backlight boost)</t>
+  </si>
+  <si>
+    <t>C86659</t>
   </si>
 </sst>
 </file>
@@ -898,10 +904,13 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="17" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="42">
@@ -1224,7 +1233,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D38"/>
+  <dimension ref="A1:D39"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
     <col min="1" max="1" width="32.62890625" customWidth="1"/>
@@ -1275,7 +1284,7 @@
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A4" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="B4" t="s">
         <v>11</v>
@@ -1289,10 +1298,10 @@
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A5" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="B5" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
       <c r="C5" t="s">
         <v>6</v>
@@ -1303,7 +1312,7 @@
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A6" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="B6" t="s">
         <v>14</v>
@@ -1317,7 +1326,7 @@
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A7" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="B7" t="s">
         <v>16</v>
@@ -1331,10 +1340,10 @@
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A8" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="B8" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="C8" t="s">
         <v>6</v>
@@ -1359,7 +1368,7 @@
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A10" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="B10" t="s">
         <v>22</v>
@@ -1373,10 +1382,10 @@
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A11" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="B11" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="C11" t="s">
         <v>6</v>
@@ -1387,10 +1396,10 @@
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A12" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="B12" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="C12" t="s">
         <v>25</v>
@@ -1401,10 +1410,10 @@
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A13" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="B13" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="C13" t="s">
         <v>27</v>
@@ -1415,7 +1424,7 @@
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A14" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="B14" t="s">
         <v>29</v>
@@ -1429,7 +1438,7 @@
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A15" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="B15" t="s">
         <v>31</v>
@@ -1454,7 +1463,7 @@
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A17" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="B17" t="s">
         <v>35</v>
@@ -1468,7 +1477,7 @@
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A18" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="B18" t="s">
         <v>37</v>
@@ -1482,7 +1491,7 @@
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A19" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="B19" t="s">
         <v>40</v>
@@ -1496,262 +1505,273 @@
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A20" t="s">
-        <v>109</v>
+        <v>132</v>
       </c>
       <c r="B20" t="s">
         <v>43</v>
       </c>
-      <c r="C20" t="s">
-        <v>44</v>
+      <c r="C20" s="2">
+        <v>5020</v>
       </c>
       <c r="D20" t="s">
-        <v>45</v>
+        <v>133</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A21" s="1" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="B21" t="s">
+        <v>44</v>
+      </c>
+      <c r="C21" t="s">
+        <v>45</v>
+      </c>
+      <c r="D21" t="s">
         <v>46</v>
-      </c>
-      <c r="C21" t="s">
-        <v>47</v>
-      </c>
-      <c r="D21" t="s">
-        <v>48</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A22" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="B22" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="C22" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="D22" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A23" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="B23" t="s">
+        <v>49</v>
+      </c>
+      <c r="C23" t="s">
+        <v>50</v>
+      </c>
+      <c r="D23" t="s">
         <v>51</v>
-      </c>
-      <c r="C23" t="s">
-        <v>52</v>
-      </c>
-      <c r="D23" t="s">
-        <v>53</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A24" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="B24" t="s">
+        <v>52</v>
+      </c>
+      <c r="C24" t="s">
+        <v>53</v>
+      </c>
+      <c r="D24" t="s">
         <v>54</v>
-      </c>
-      <c r="C24" t="s">
-        <v>55</v>
-      </c>
-      <c r="D24" t="s">
-        <v>56</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A25" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="B25" t="s">
+        <v>55</v>
+      </c>
+      <c r="C25" t="s">
+        <v>56</v>
+      </c>
+      <c r="D25" t="s">
         <v>57</v>
-      </c>
-      <c r="C25" t="s">
-        <v>58</v>
-      </c>
-      <c r="D25" t="s">
-        <v>59</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A26" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="B26" t="s">
+        <v>58</v>
+      </c>
+      <c r="C26" t="s">
+        <v>59</v>
+      </c>
+      <c r="D26" t="s">
         <v>60</v>
-      </c>
-      <c r="C26" t="s">
-        <v>61</v>
-      </c>
-      <c r="D26" t="s">
-        <v>62</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A27" s="1" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="B27" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="C27" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="D27" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A28" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="B28" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="C28" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="D28" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A29" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="B29" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="C29" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="D29" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A30" t="s">
+        <v>66</v>
+      </c>
+      <c r="B30" t="s">
+        <v>67</v>
+      </c>
+      <c r="D30" t="s">
         <v>68</v>
-      </c>
-      <c r="B30" t="s">
-        <v>69</v>
-      </c>
-      <c r="D30" t="s">
-        <v>70</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A31" s="1" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="B31" t="s">
+        <v>69</v>
+      </c>
+      <c r="C31" t="s">
+        <v>70</v>
+      </c>
+      <c r="D31" t="s">
         <v>71</v>
-      </c>
-      <c r="C31" t="s">
-        <v>72</v>
-      </c>
-      <c r="D31" t="s">
-        <v>73</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A32" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="B32" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="D32" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A33" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="B33" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="C33" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="D33" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A34" s="1" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="B34" t="s">
+        <v>76</v>
+      </c>
+      <c r="C34" t="s">
+        <v>77</v>
+      </c>
+      <c r="D34" t="s">
         <v>78</v>
-      </c>
-      <c r="C34" t="s">
-        <v>79</v>
-      </c>
-      <c r="D34" t="s">
-        <v>80</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A35" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="B35" t="s">
+        <v>79</v>
+      </c>
+      <c r="C35" t="s">
+        <v>80</v>
+      </c>
+      <c r="D35" t="s">
         <v>81</v>
-      </c>
-      <c r="C35" t="s">
-        <v>82</v>
-      </c>
-      <c r="D35" t="s">
-        <v>83</v>
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A36" t="s">
-        <v>98</v>
+        <v>130</v>
       </c>
       <c r="B36" t="s">
-        <v>84</v>
-      </c>
-      <c r="C36" t="s">
-        <v>85</v>
+        <v>129</v>
       </c>
       <c r="D36" t="s">
-        <v>86</v>
+        <v>131</v>
       </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A37" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="B37" t="s">
-        <v>87</v>
+        <v>82</v>
       </c>
       <c r="C37" t="s">
-        <v>88</v>
+        <v>83</v>
       </c>
       <c r="D37" t="s">
-        <v>89</v>
+        <v>84</v>
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A38" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="B38" t="s">
-        <v>90</v>
+        <v>85</v>
       </c>
       <c r="C38" t="s">
+        <v>86</v>
+      </c>
+      <c r="D38" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+      <c r="A39" t="s">
+        <v>98</v>
+      </c>
+      <c r="B39" t="s">
+        <v>88</v>
+      </c>
+      <c r="C39" t="s">
+        <v>89</v>
+      </c>
+      <c r="D39" t="s">
         <v>91</v>
-      </c>
-      <c r="D38" t="s">
-        <v>93</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update files for 3D printed case
</commit_message>
<xml_diff>
--- a/pcb/esp32p4/mainboard/pcb assembly JLC/p2_pcb_esp32p4_v1_4_bom_JLC.xlsx
+++ b/pcb/esp32p4/mainboard/pcb assembly JLC/p2_pcb_esp32p4_v1_4_bom_JLC.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="151" uniqueCount="134">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="153" uniqueCount="136">
   <si>
     <t>Comment</t>
   </si>
@@ -421,6 +421,12 @@
   </si>
   <si>
     <t>C86659</t>
+  </si>
+  <si>
+    <t>C280582</t>
+  </si>
+  <si>
+    <t>C2886897</t>
   </si>
 </sst>
 </file>
@@ -1233,7 +1239,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D39"/>
+  <dimension ref="A1:E39"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
     <col min="1" max="1" width="32.62890625" customWidth="1"/>
@@ -1461,7 +1467,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A17" t="s">
         <v>119</v>
       </c>
@@ -1475,7 +1481,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A18" t="s">
         <v>108</v>
       </c>
@@ -1489,7 +1495,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A19" t="s">
         <v>107</v>
       </c>
@@ -1503,7 +1509,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A20" t="s">
         <v>132</v>
       </c>
@@ -1516,8 +1522,11 @@
       <c r="D20" t="s">
         <v>133</v>
       </c>
-    </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+      <c r="E20" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A21" s="1" t="s">
         <v>106</v>
       </c>
@@ -1531,7 +1540,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A22" t="s">
         <v>105</v>
       </c>
@@ -1545,7 +1554,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A23" t="s">
         <v>104</v>
       </c>
@@ -1559,7 +1568,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A24" t="s">
         <v>103</v>
       </c>
@@ -1573,7 +1582,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A25" t="s">
         <v>102</v>
       </c>
@@ -1587,7 +1596,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A26" t="s">
         <v>101</v>
       </c>
@@ -1601,7 +1610,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A27" s="1" t="s">
         <v>122</v>
       </c>
@@ -1615,7 +1624,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A28" t="s">
         <v>100</v>
       </c>
@@ -1629,7 +1638,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A29" t="s">
         <v>121</v>
       </c>
@@ -1643,7 +1652,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A30" t="s">
         <v>66</v>
       </c>
@@ -1654,7 +1663,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A31" s="1" t="s">
         <v>99</v>
       </c>
@@ -1668,7 +1677,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A32" t="s">
         <v>92</v>
       </c>
@@ -1679,7 +1688,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A33" t="s">
         <v>93</v>
       </c>
@@ -1693,7 +1702,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A34" s="1" t="s">
         <v>94</v>
       </c>
@@ -1707,7 +1716,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A35" t="s">
         <v>95</v>
       </c>
@@ -1721,7 +1730,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A36" t="s">
         <v>130</v>
       </c>
@@ -1732,7 +1741,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A37" t="s">
         <v>96</v>
       </c>
@@ -1746,7 +1755,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+    <row r="38" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A38" t="s">
         <v>97</v>
       </c>
@@ -1760,7 +1769,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+    <row r="39" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A39" t="s">
         <v>98</v>
       </c>
@@ -1772,6 +1781,9 @@
       </c>
       <c r="D39" t="s">
         <v>91</v>
+      </c>
+      <c r="E39" t="s">
+        <v>135</v>
       </c>
     </row>
   </sheetData>

</xml_diff>